<commit_message>
Solved format issue with timeslots (from int to string)
</commit_message>
<xml_diff>
--- a/data/example_entry.xlsx
+++ b/data/example_entry.xlsx
@@ -79,10 +79,10 @@
     <t>false</t>
   </si>
   <si>
-    <t>1,2,3,4,5,6,7</t>
-  </si>
-  <si>
-    <t>1,2,3,4,5</t>
+    <t>Mo1,Mo2,Mo3,Mo4,Mo5,Mo6,Di1</t>
+  </si>
+  <si>
+    <t>Mo1,Mo2,Mo3,Mo4,Mo5</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
First test run serving as proof of concept. Just three teachers and one class easy to handle.
</commit_message>
<xml_diff>
--- a/data/example_entry.xlsx
+++ b/data/example_entry.xlsx
@@ -1,118 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robin\OneDrive\Desktop\Timetable\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81CDAA2-7DA7-47A7-A587-DA997A4ECFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="9210" windowWidth="27320" windowHeight="9830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4290" yWindow="9210" windowWidth="27320" windowHeight="9830" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>subjects</t>
-  </si>
-  <si>
-    <t>max_weekly_hours</t>
-  </si>
-  <si>
-    <t>availability</t>
-  </si>
-  <si>
-    <t>role</t>
-  </si>
-  <si>
-    <t>is_homeroom_teacher</t>
-  </si>
-  <si>
-    <t>homeroom_class</t>
-  </si>
-  <si>
-    <t>frabai</t>
-  </si>
-  <si>
-    <t>Franziska Baißbiel</t>
-  </si>
-  <si>
-    <t>Deutsch,Mathe,Sport</t>
-  </si>
-  <si>
-    <t>full_teacher</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>1a</t>
-  </si>
-  <si>
-    <t>balu</t>
-  </si>
-  <si>
-    <t>Basel Lula</t>
-  </si>
-  <si>
-    <t>Mathe,Geographie,Geschichte</t>
-  </si>
-  <si>
-    <t>part_time</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>Mo1,Mo2,Mo3,Mo4,Mo5,Mo6,Di1</t>
-  </si>
-  <si>
-    <t>Mo1,Mo2,Mo3,Mo4,Mo5</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -135,34 +62,93 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -450,95 +436,173 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col width="15.453125" bestFit="1" customWidth="1" min="1" max="2"/>
+    <col width="26.54296875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="15.81640625" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
+    <col width="18.81640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="13.54296875" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="18.81640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="14.54296875" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>subjects</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>max_weekly_hours</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>is_homeroom_teacher</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>homeroom_class</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>frabai</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Franziska Baißbiel</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Deutsch,Mathe,Sport</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Mo1,Mo2,Mo3,Mo4,Mo5,Mo6,Di1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>full_teacher</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>balu</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Basel Lula</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mathe,Geographie,Geschichte</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
-        <v>13</v>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Mo1,Mo2,Mo3,Mo4,Mo5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>part_time</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="4">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rosa</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Robin Salzmann</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Geschichte,MNK,Sport</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mo1,Mo2,Mo3,Mo4,Mo5,Mo6,Di1,Di2,Di3,Di4,Di5,Di6,Mi1,Mi2,Mi3,Mi4,Mi5,Mi6,Do1,Do2,Do3,Do4,Do5,Do6,Fr1,Fr2,Fr3,Fr4,Fr5,Fr6,MoNU,DiNU,MiNU,DoNU,FrNU</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>full_teacher</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plan will not be created from scratch but modeled according to older version - this might not yet work properly. Listing of subjects has been removed from output format. README.md update to include distr and deployment info.
</commit_message>
<xml_diff>
--- a/data/example_entry.xlsx
+++ b/data/example_entry.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="classes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="required_hours" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -852,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -861,11 +862,6 @@
           <t>class_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>required_subjects</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -873,11 +869,6 @@
           <t>1a</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>D:6,M/LB:2,SU:3,M:4,BK:1,Mus:1,Sp:2,D/L:1</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -885,11 +876,6 @@
           <t>1b</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>D:6,M/LB:2,SU:3,M:4,BK:1,Mus:1,Sp:2,D/L:1</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -897,11 +883,6 @@
           <t>2a</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>TW:1,D:7,D/L:1,M:6,BK:1,SU:2,Sp:2,Mus:1,Rel:2</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -909,11 +890,6 @@
           <t>2b</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>TW:1,D:7,D/L:1,M:6,BK:1,SU:2,Sp:2,Mus:1,Rel:2</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -921,11 +897,6 @@
           <t>3a</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>M:4,D:4,D/L:2,E:2,BK:1,Mus:2,Rel:2,TW:1,Sp:2,SU:2</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -933,11 +904,6 @@
           <t>3b</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>M:4,D:4,D/L:2,E:2,BK:1,Mus:2,Rel:2,TW:1,Sp:2,SU:2</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -945,11 +911,6 @@
           <t>4a</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>D:5,D/L:2,M:6,Sp:2,E:2,BK:1,TW:1,Rel:2,Mus:2,SU:2</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -957,10 +918,591 @@
           <t>4b</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>grade</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>subject</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>M/LB</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SU</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mus</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sp</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>D:5,D/L:2,M:6,Sp:2,E:2,BK:1,TW:1,Rel:2,Mus:2,SU:2</t>
-        </is>
+          <t>D/L</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>D/L</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SU</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sp</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mus</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Rel</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>D/L</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mus</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Rel</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sp</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SU</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>D/L</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sp</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Rel</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mus</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SU</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>